<commit_message>
integration with loan application system
</commit_message>
<xml_diff>
--- a/public/templates/group_loans.xlsx
+++ b/public/templates/group_loans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp1\htdocs\uwz\uwz\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF6A92D-657F-4D56-B82C-167F447D0B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECA9506-CB74-4F25-BF9B-FF8BE3D2E546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8AE6995C-61F6-4426-AE54-050AF86B364A}"/>
   </bookViews>
@@ -34,82 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
-  <si>
-    <t>New</t>
-  </si>
-  <si>
-    <t>financed</t>
-  </si>
-  <si>
-    <t>Resubmission</t>
-  </si>
-  <si>
-    <t>Phase 1</t>
-  </si>
-  <si>
-    <t>Phase 2</t>
-  </si>
-  <si>
-    <t>Phase 3</t>
-  </si>
-  <si>
-    <t>MZAWO WOMEN GROUP</t>
-  </si>
-  <si>
-    <t>001</t>
-  </si>
-  <si>
-    <t>WIKWATYO WOMEN GRP</t>
-  </si>
-  <si>
-    <t>002</t>
-  </si>
-  <si>
-    <t>DISCOVERY YOUTH GRP</t>
-  </si>
-  <si>
-    <t>003</t>
-  </si>
-  <si>
-    <t>MWANEDU SHG</t>
-  </si>
-  <si>
-    <t>004</t>
-  </si>
-  <si>
-    <t>KILIMO NI BORA W.G.</t>
-  </si>
-  <si>
-    <t>005</t>
-  </si>
-  <si>
-    <t>Refinancing</t>
-  </si>
-  <si>
-    <t>Reallocation</t>
-  </si>
-  <si>
-    <t>001/001</t>
-  </si>
-  <si>
-    <t>001/002</t>
-  </si>
-  <si>
-    <t>001/003</t>
-  </si>
-  <si>
-    <t>001/005</t>
-  </si>
-  <si>
-    <t>001/006</t>
-  </si>
-  <si>
-    <t>cancelled</t>
-  </si>
-  <si>
-    <t>null</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>S/No.*</t>
   </si>
@@ -568,307 +493,97 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="11">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="3">
-        <v>42013</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="5">
-        <v>100000</v>
-      </c>
-      <c r="J2" s="5">
-        <v>100000</v>
-      </c>
-      <c r="K2" s="5">
-        <v>100000</v>
-      </c>
-      <c r="L2" s="5">
-        <v>56600</v>
-      </c>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="11">
-        <v>2</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3">
-        <v>42033</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="5">
-        <v>100000</v>
-      </c>
-      <c r="J3" s="5">
-        <v>100000</v>
-      </c>
-      <c r="K3" s="5">
-        <v>80000</v>
-      </c>
-      <c r="L3" s="5">
-        <v>100000</v>
-      </c>
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="11">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3">
-        <v>42013</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="5">
-        <v>100000</v>
-      </c>
-      <c r="J4" s="5">
-        <v>100000</v>
-      </c>
-      <c r="K4" s="5">
-        <v>100000</v>
-      </c>
-      <c r="L4" s="5">
-        <v>73100</v>
-      </c>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="11">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5" s="5">
-        <v>100000</v>
-      </c>
-      <c r="J5" s="5">
-        <v>100000</v>
-      </c>
-      <c r="K5" s="5">
-        <v>0</v>
-      </c>
-      <c r="L5" s="5">
-        <v>0</v>
-      </c>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="11">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3">
-        <v>42013</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="5">
-        <v>100000</v>
-      </c>
-      <c r="J6" s="5">
-        <v>1000000</v>
-      </c>
-      <c r="K6" s="5">
-        <v>70000</v>
-      </c>
-      <c r="L6" s="5">
-        <v>49000</v>
-      </c>
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="11">
-        <v>6</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3">
-        <v>42013</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="5">
-        <v>400000</v>
-      </c>
-      <c r="J7" s="5">
-        <v>200000</v>
-      </c>
-      <c r="K7" s="5">
-        <v>200000</v>
-      </c>
-      <c r="L7" s="5">
-        <v>100000</v>
-      </c>
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A8" s="11">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" s="5">
-        <v>200000</v>
-      </c>
-      <c r="J8" s="5">
-        <v>200000</v>
-      </c>
-      <c r="K8" s="5">
-        <v>0</v>
-      </c>
-      <c r="L8" s="5">
-        <v>0</v>
-      </c>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>